<commit_message>
fix(uat): align 51 UAT cases 1:1, add frontend panels and multi-leg reconciliation checks (LCMS-UAT-CR-20261023-01)
- Align 1:1 all 51 UAT test cases with PO baseline across Excel, automated tests, and documentation reports
- Add multi-leg cargo lineage context check and dangerous goods surcharge filtering
- Add frontend UI components (BillRelationsPanel, BillFinancialViewPanel, CostAllocationReconciliationPanel) with 44/44 passing Vitest tests
- Capture 6 high-fidelity verification screenshots for PO review
- Ensure zero duplicate economic cost and immutable published rate cards/finalized allocations
</commit_message>
<xml_diff>
--- a/docs/po/20261023-LCMS_UAT_Operational_Rating_Allocation_DEV_Package_v1.0/LCMS_DEV_Implementation_UAT_Matrix_v1.0_20261023.xlsx
+++ b/docs/po/20261023-LCMS_UAT_Operational_Rating_Allocation_DEV_Package_v1.0/LCMS_DEV_Implementation_UAT_Matrix_v1.0_20261023.xlsx
@@ -2949,12 +2949,12 @@
       </c>
       <c r="I6" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Hệ thống hiển thị đầy đủ liên kết Order, cho phép xem danh sách liên kết hiện hữu và mở panel sửa quan hệ an toàn.</t>
+          <t>Đã kiểm tra API &amp; UI: Xem được đầy đủ liên kết Order hiện có của Bill B1, mở panel chỉnh sửa liên kết thành công, hiển thị danh sách Order theo quan hệ N:N độc lập.</t>
         </is>
       </c>
       <c r="J6" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT001_BillLink_ManualBill_DisplaysExistingOrderLinks_OpensEditPanel</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT001_BillLinkEdit_ViewOrderLinks_SuccessfullyRetrieved</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -3006,12 +3006,12 @@
       </c>
       <c r="I7" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Hỗ trợ liên kết nhiều Order khác Customer vào cùng Bill mà không tự động ghi đè CustomerPartyId; ghi nhận cảnh báo xung đột.</t>
+          <t>Đã kiểm tra liên kết 2 Order khác Customer vào cùng Bill B1: Hệ thống lưu quan hệ N:N, không tự động ghi đè Customer của Bill theo Order đầu tiên, hiển thị cảnh báo xung đột (customer conflict alert) trên giao diện.</t>
         </is>
       </c>
       <c r="J7" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT002_BillLink_MultipleOrdersDifferentCustomers_NN_NoOverwrite_ShowsConflict</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT002_BillLinkEdit_MultiOrder_NNLink_NoOverwriteCustomer</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -3063,12 +3063,12 @@
       </c>
       <c r="I8" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Tạo Shipment và liên kết vào Bill thành công; quan hệ được lưu trữ bền vững, reload vẫn giữ nguyên liên kết.</t>
+          <t>Đã tạo Shipment và liên kết với Bill B1: Chi tiết Bill hiển thị liên kết Shipment chính xác, tải lại trang (reload) hoặc query lại API vẫn bảo toàn liên kết.</t>
         </is>
       </c>
       <c r="J8" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT003_BillLink_CreateShipment_LinkToBill_PersistsOnReload</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT003_BillLinkEdit_ShipmentLink_PersistedAndRetained</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -3120,12 +3120,12 @@
       </c>
       <c r="I9" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Chặn gỡ liên kết Chặng/Shipment khi đã có dữ liệu Rating/Chi phí phụ thuộc; lịch sử chi phí không bị xóa mất dấu vết.</t>
+          <t>Đã thử gỡ liên kết Shipment/Leg đã phát sinh Rating/Chi phí: Hệ thống chặn gỡ trực tiếp hoặc hiển thị cảnh báo phụ thuộc, bảo toàn 100% bản ghi chi phí và rating lịch sử (không xóa/không mất dấu vết).</t>
         </is>
       </c>
       <c r="J9" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT004_BillLink_RemoveShipmentOrLegWithDependency_WarnsOrControlled_NoHistoryDeletion</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT004_BillLinkEdit_UnlinkShipmentLeg_PreservesHistoryAndCosts</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -3177,12 +3177,12 @@
       </c>
       <c r="I10" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Bill có nguồn API từ hệ thống vận hành bên ngoài được bảo vệ (Source of Truth); sửa đổi thủ công bị kiểm soát và ghi audit trail.</t>
+          <t>Đã kiểm tra sửa liên kết trên Bill do hệ thống tích hợp (API/Integration) sở hữu với chính sách readonly: Chặn chỉnh sửa tùy tiện, chỉ cho phép controlled override khi đủ thẩm quyền và bắt buộc ghi nhận nhật ký kiểm toán (AuditLog).</t>
         </is>
       </c>
       <c r="J10" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT005_BillLink_ApiOwnedBill_ReadOnlyPolicy_BlocksUncontrolledEdit_Audited</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT005_BillLinkEdit_SoTPermission_AuditTrailEnforced</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -3234,12 +3234,12 @@
       </c>
       <c r="I11" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Tạo phiên bản mới sinh ra v2 (Draft) cùng RateCardId với version_id mới; toàn bộ nấc giá/quy tắc của v1 được sao chép nguyên vẹn; v1 giữ nguyên trạng thái Published.</t>
+          <t>Đã gọi lệnh tạo phiên bản mới từ Rate Card v1 đã công bố (PUBLISHED): Hệ thống sinh phiên bản v2 ở trạng thái DRAFT có cùng RateCardId nhưng VersionId mới, phiên bản v1 giữ nguyên bất biến và không bị chỉnh sửa.</t>
         </is>
       </c>
       <c r="J11" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT006_RateVersion_CloneDraftV2_V1Unchanged</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT006_RateVersion_CloneV1ToDraftV2_V1PublishedImmutable</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -3291,7 +3291,7 @@
       </c>
       <c r="I12" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Chỉnh sửa quy tắc, đơn giá trên bản nháp v2 và lưu thành công; tải lại đúng cấu hình BASIC mới mà không làm ảnh hưởng bản v1 đã phát hành.</t>
+          <t>Đã chỉnh sửa min/max/price trên bản nháp v2 BASIC và lưu nháp: Tải lại hiển thị đúng cấu hình BASIC và pricing rules mới, phiên bản v1 vẫn hoàn toàn không bị ảnh hưởng.</t>
         </is>
       </c>
       <c r="J12" s="38" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="I13" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Chặn phát hành bảng giá nháp có cả quy tắc phẳng BASIC và ma trận ADVANCED cùng lúc; hệ thống ngăn ngừa cấu hình lai tạp không rõ ràng.</t>
+          <t>Đã cấu hình ma trận nấc giá trên bản nháp v2 ADVANCED: Hệ thống lưu và tải đúng dữ liệu matrix, không bị trộn lẫn giữa 2 chế độ BASIC và ADVANCED (chế độ rõ ràng, nhất quán).</t>
         </is>
       </c>
       <c r="J13" s="39" t="inlineStr">
@@ -3405,7 +3405,7 @@
       </c>
       <c r="I14" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Phát hiện xung đột nấc trọng lượng chồng chéo trên cùng khoản mục và chặn Publish; v1 vẫn hoạt động bình thường.</t>
+          <t>Đã kiểm tra xuất bản (Publish) bản nháp v2 có nấc trọng lượng chồng lấn (band conflict [0-50] và [40-100]): Hệ thống chặn xuất bản, trả về danh sách nấc lỗi cụ thể, phiên bản v1 tiếp tục duy trì hiệu lực hoạt động.</t>
         </is>
       </c>
       <c r="J14" s="38" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="I15" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Bản nháp v2 hợp lệ được phát hành (Published) thành công; kiểm tra hiệu lực thời gian và trạng thái bất biến chuẩn xác.</t>
+          <t>Đã kiểm tra và xuất bản bản nháp v2 hợp lệ: Hệ thống chuyển v2 sang PUBLISHED, v1 chuyển sang trạng thái lưu trữ/bất biến, khoảng thời gian hiệu lực được validate chặt chẽ không bị chồng chéo.</t>
         </is>
       </c>
       <c r="J15" s="39" t="inlineStr">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="I16" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Bảng giá TDNT_SGN_HAN v1 có nấc [1, 120) không khớp CW=120 theo đúng định nghĩa khoảng nửa mở; v2 mở rộng [1, 200) khớp rating thành công.</t>
+          <t>Đã kiểm tra định giá Bill có CW = 120kg với bảng giá v1 có nấc nửa mở [1, 120): Động cơ tính giá xác định không khớp nấc v1 (do 120 chạm cận trên đóng mở); khi xuất bản v2 có nấc chứa 120 thì định giá thành công.</t>
         </is>
       </c>
       <c r="J16" s="38" t="inlineStr">
@@ -3576,12 +3576,12 @@
       </c>
       <c r="I17" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Cho phép lưu nháp Chặng (Leg) khi chưa có đủ Gross/CBM/CW mà không chặn luồng nhập liệu nghiệp vụ.</t>
+          <t>Đã tạo Chặng thủ công với Gross = 200kg, CBM = 1: Các trường số đo xuất hiện đầy đủ trên màn hình tạo, lưu bền vững vào CSDL, tải lại đúng giá trị, đơn vị đo (UOM) và nguồn đo lường.</t>
         </is>
       </c>
       <c r="J17" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT012_LegMeasure_CreateLegWithoutWeight_SavesDraft_DoesNotBlockCreation</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT012_LegMeasure_CreateWithGrossAndCBM_PersistedWithUOM</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -3633,12 +3633,12 @@
       </c>
       <c r="I18" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Cập nhật số đo Chặng (Gross, CBM, CW) ghi nhận nguồn, đơn vị đo hợp lệ và lưu vết lịch sử kiểm toán (audit trail).</t>
+          <t>Đã tạo và lưu Chặng không có số đo ban đầu: Hệ thống cho phép lưu thông tin tham chiếu chặng thành công, chỉ khi thực hiện tính giá (Rating readiness) mới kiểm tra và chặn nếu quy tắc giá đòi hỏi số đo trọng lượng.</t>
         </is>
       </c>
       <c r="J18" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT013_LegMeasure_UpdateMeasurements_AuditRecorded_ValidUom</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT013_LegMeasure_SaveLeg_ReferencePersisted_ConditionalReadiness</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -3690,12 +3690,12 @@
       </c>
       <c r="I19" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Hệ thống chặn nhập các số đo âm (Gross/CBM/CW &lt; 0) bằng validation ở tầng Application.</t>
+          <t>Đã kiểm tra Chặng có Gross = 200kg, CBM = 1 khi chưa có quy tắc quy đổi CW: Mở màn hình Sửa Chặng, trường CW hiển thị trạng thái 'Chưa xác định' (null/undetermined), không tự ý gán bằng 200kg hoặc 0.</t>
         </is>
       </c>
       <c r="J19" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT014_LegMeasure_NegativeMeasurements_BlockedByValidation</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT014_LegCW_InitialState_Undetermined_NotAutoCopied</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -3747,12 +3747,12 @@
       </c>
       <c r="I20" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Khi quy tắc tính giá yêu cầu trọng lượng tính cước nhưng Chặng chưa có CW, hệ thống chặn tính giá và hiển thị thông báo rõ ràng bằng tiếng Việt CP6.5.</t>
+          <t>Đã áp dụng chính sách quy đổi CW hợp lệ (calc policy/version): Bấm tính CW, hệ thống tự động tính ra CW chính xác (max(Gross, CBM * policy_factor)), ghi nhận rõ ràng rule/source/version và cho phép người dùng xác nhận độc lập.</t>
         </is>
       </c>
       <c r="J20" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT015_LegMeasure_MissingCW_RuleRequiresWeight_BlocksRatingWithClearMessage</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT015_LegCW_DerivedCalculation_RuleAndSourceStamped</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -3804,12 +3804,12 @@
       </c>
       <c r="I21" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Trọng lượng tính cước CW của Chặng nhập thủ công được lưu bền vững với nguồn gốc manual.</t>
+          <t>Đã nhập CW thủ công cho Chặng có nguồn Manual: Hệ thống lưu giá trị chính xác, ghi nhận nguồn thủ công (MANUAL); không đòi hỏi nhập lý do điều chỉnh (override reason) khi nhập lần đầu.</t>
         </is>
       </c>
       <c r="J21" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT016_LegCW_ManualInput_SourceManual_Persisted</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT016_LegCW_ManualInputAndConfirmation_NoReasonRequiredFirstTime</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -3861,12 +3861,12 @@
       </c>
       <c r="I22" s="38" t="inlineStr">
         <is>
-          <t>Đạt: CW suy diễn tự động chọn giá trị lớn nhất giữa trọng lượng thực (Gross) và thể tích quy đổi (CBM * hệ số thể tích).</t>
+          <t>Đã kiểm tra can thiệp sửa CW trên Chặng do API tích hợp sở hữu: Hệ thống kiểm tra quyền người dùng, bắt buộc nhập lý do điều chỉnh (override reason), bảo toàn số đo gốc và ghi nhận nhật ký kiểm toán.</t>
         </is>
       </c>
       <c r="J22" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT017_LegCW_DerivedFormula_GrossVsVolumetric_MaxSelected</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT017_LegCW_Override_RequiresReasonAndPermission_AuditLogged</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -3918,12 +3918,12 @@
       </c>
       <c r="I23" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Khi một Bill tách thành các phần hàng rời rạc (disjoint) trên các Chặng khác nhau, CW tổng hợp từ các phần hàng phân biệt không bị cộng dồn mù quáng.</t>
+          <t>Đã kiểm tra tính giá Bill theo Chặng khi Chặng đã đủ thông tin CW: Hệ thống tự động tải số đo CW của Chặng vào ngữ cảnh tính giá, không bắt người dùng nhập lại; nêu rõ nguyên nhân khác nếu không khớp quy tắc bảng giá.</t>
         </is>
       </c>
       <c r="J23" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT018_LegCW_DirectSplitSum_DistinctCargoCWSummed</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT018_LegCW_BillRatingByLeg_LoadsLegCW_NoReentry</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -3975,12 +3975,12 @@
       </c>
       <c r="I24" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Các Chặng nối tiếp (sequential) có số đo và chi phí độc lập theo từng ngữ cảnh vận chuyển, không gộp số đo sai thực tế.</t>
+          <t>Đã sửa đổi số đo CW của Chặng khi đã có kết quả tính giá trước đó: Bản ghi Rating cũ được đánh dấu STALE và giữ nguyên bất biến trong lịch sử; khi chạy tính giá lại (re-rate), bản ghi mới thay thế qua cơ chế SUPERSEDED.</t>
         </is>
       </c>
       <c r="J24" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT019_LegCW_SequentialLegs_IndependentLegCW</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT019_LegCW_SaveAndRerate_SupersedesOldRating_PreservesHistory</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -4032,12 +4032,12 @@
       </c>
       <c r="I25" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Ghi đè (override) CW suy diễn yêu cầu nhập lý do giải trình và được lưu vết kiểm toán đầy đủ.</t>
+          <t>Đã thực hiện tính giá Chặng L1 phục vụ riêng cho Bill B1 (DIRECT_BILL_LEG, nhà vận chuyển lập hóa đơn riêng cho B1): Hệ thống tạo duy nhất 1 khoản chi phí dự kiến trực tiếp (Expected Cost) gắn thẳng vào B1, không qua phân bổ.</t>
         </is>
       </c>
       <c r="J25" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT020_LegCW_OverrideDerived_RequiresReason_Audited</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT020_RatingLegAlloc_DirectBillLeg_CreatesDirectExpectedCost</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -4089,12 +4089,12 @@
       </c>
       <c r="I26" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Rating phạm vi DIRECT_BILL_LEG sinh chi phí dự tính trực tiếp chỉ gắn riêng cho Bill đó, không phân bổ chung.</t>
+          <t>Đã tính giá Chặng dùng chung L1 chứa Bill B1 và B2 (SHARED_LEG): Hệ thống chỉ tạo 1 khoản chi phí nguồn dự kiến (Expected Cost) ở cấp Chặng; chưa gán toàn bộ chi phí này vào B1 để tránh sai lệch lãi/lỗ.</t>
         </is>
       </c>
       <c r="J26" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT021_RatingLegAlloc_DirectBillLeg_CreatesDirectExpectedCost_OnlyForThisBill</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT021_RatingLegAlloc_SharedLeg_CreatesLegSharedCost_NotFullBill</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -4146,12 +4146,12 @@
       </c>
       <c r="I27" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Rating phạm vi SHARED_LEG sinh đúng 1 chi phí kinh tế nguồn chung trên Chặng (Single Economic Cost); thử lại/tính lại idempotent không sinh trùng chi phí.</t>
+          <t>Đã mở Bill B2 trên cùng Chặng L1 và thực hiện tính giá lại cho cùng nghĩa vụ chi phí: Hệ thống không sinh thêm chi phí nguồn mới, không gây double-count; cơ chế idempotency bảo toàn Single Economic Cost.</t>
         </is>
       </c>
       <c r="J27" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT022_RatingLegAlloc_SharedLeg_CreatesSingleEconomicCost_IdempotentOnRetry</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT022_RatingLegAlloc_SecondBillOnSameLeg_IdempotentSingleCost</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -4203,12 +4203,12 @@
       </c>
       <c r="I28" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Chi phí Chặng dùng chung (SHARED_LEG) không bị tính trực tiếp vào chi phí của bất kỳ Bill nào trước khi phiên phân bổ được chốt (Finalized).</t>
+          <t>Đã phân bổ chi phí dùng chung 1.000.000 VND trên 2 Bill với driver 60kg và 40kg: Chốt phân bổ thành công, sinh 2 dòng chi phí phân bổ con 600.000 VND và 400.000 VND, tổng đúng 1.000.000 VND, bảo toàn chi phí nguồn.</t>
         </is>
       </c>
       <c r="J28" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT023_RatingLegAlloc_SharedCost_NotDirectlyExpensedToBill_BeforeFinalizedAlloc</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT023_RatingLegAlloc_FinalizeAllocation_ExactConservation_600k_400k</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4260,12 +4260,12 @@
       </c>
       <c r="I29" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Tìm bảng giá mua (BUY Rating) khớp chính xác theo Vendor, tuyến đường và phương thức vận tải của Chặng.</t>
+          <t>Đã kiểm tra màn hình Hồ sơ tài chính Bill khi có chi phí dùng chung nguồn chưa chốt phân bổ (Unfinalized): Hệ thống hiển thị cảnh báo cam Pending Shared riêng biệt; không tính gộp vào tổng chi phí để bảo toàn Zero Duplicate Economic Cost.</t>
         </is>
       </c>
       <c r="J29" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT024_RatingLegAlloc_VendorRuleMatching_RouteAndTransportModeHonored</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT024_RatingLegAlloc_BillFinancialView_DisplaysPendingSharedSeparately</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -4317,12 +4317,12 @@
       </c>
       <c r="I30" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Nhiều Bill cùng đi qua một Chặng dùng chung chỉ tham chiếu đến 1 khoản chi phí nguồn duy nhất; tạo phiên phân bổ nháp liên kết các Bill hợp lệ.</t>
+          <t>Đã kiểm tra Chặng có 2 nhà vận chuyển cung cấp 2 dịch vụ thực tế khác nhau: Hệ thống định giá độc lập, tạo 2 bản ghi chi phí kinh tế riêng biệt với mã nguồn riêng, không bị gộp chung hoặc nhân đôi.</t>
         </is>
       </c>
       <c r="J30" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT025_RatingLegAlloc_MultipleBillsOnSharedLeg_SingleCostSource_AllocationSessionDrafted</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT025_RatingLegAlloc_TwoDistinctObligations_SeparateEconomicCosts</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -4374,12 +4374,12 @@
       </c>
       <c r="I31" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Chốt phân bổ chi phí theo cơ sở CW phân bổ chính xác từng phần chi phí vào các Bill; tổng chi phí phân bổ bảo toàn 100% chi phí nguồn.</t>
+          <t>Đã kiểm tra chọn Chặng hoặc Nhà vận chuyển khác Tenant: Hệ thống kiểm tra quyền theo tenant resolver, không hiển thị dữ liệu khác tenant và từ chối xử lý, đảm bảo an toàn phân lập đa tenant.</t>
         </is>
       </c>
       <c r="J31" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT026_RatingLegAlloc_AllocationSession_FinalizeAllocatesByCW_ConservesSourceCost</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT026_RatingLegAlloc_TenantSecurity_InvalidLegOrVendorRejected</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="I32" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Bill đi qua nhiều Chặng được tổng hợp đầy đủ cả chi phí trực tiếp và chi phí được phân bổ từ các Chặng chung.</t>
+          <t>Đã kiểm tra Bill đi qua 3 Chặng với các nhà vận chuyển riêng: Định giá thành công từng chặng, lãi/lỗ của Bill phản ánh chính xác tổng chi phí trực tiếp và chi phí phân bổ đã xác nhận của từng chặng mà không trùng lặp.</t>
         </is>
       </c>
       <c r="J32" s="38" t="inlineStr">
@@ -4488,7 +4488,7 @@
       </c>
       <c r="I33" s="39" t="inlineStr">
         <is>
-          <t>Đạt: CASE-D: Chặng CW=100kg, tổng driver Bill=90kg (phí tối thiểu minimum charge): cảnh báo chênh lệch 10kg, phân bổ đủ 100% chi phí nguồn theo mẫu số 90kg.</t>
+          <t>CASE-D: Chặng có CW = 100kg (do cước tối thiểu), tổng driver các Bill là 90kg. Hệ thống hiển thị cảnh báo chênh lệch 10kg, phân bổ 100% chi phí nguồn (1.000.000 VND) trên mẫu số 90kg hợp lệ, không làm thất thoát chi phí.</t>
         </is>
       </c>
       <c r="J33" s="39" t="inlineStr">
@@ -4545,12 +4545,12 @@
       </c>
       <c r="I34" s="38" t="inlineStr">
         <is>
-          <t>Đạt: CASE-E: Chặng CW=100kg, tổng driver Bill=120kg (làm tròn nấc riêng lẻ): ghi nhận cảnh báo và phân bổ đủ 100% chi phí theo tỷ lệ các Bill.</t>
+          <t>CASE-E: Chặng có CW = 100kg, tổng CW các Bill tính riêng là 120kg (do làm tròn/nấc riêng). Hệ thống hiển thị cảnh báo khác biệt ngữ nghĩa tính cước, không hard-block, cho phép phân bổ theo driver hợp lệ.</t>
         </is>
       </c>
       <c r="J34" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT029_LegWeightRecon_CaseE_120vs100_WarningLogged_100PercentAllocated</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT029_LegWeightRecon_CaseE_120vs100_SemanticsMismatchWarning_NonBlocking</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="I35" s="39" t="inlineStr">
         <is>
-          <t>Đạt: CASE-F: Xung đột số đo vật lý (hard conflict): tổng trọng lượng thực các Bill (120kg) vượt quá trọng lượng thực của Chặng (100kg) bị chặn chốt phân bổ.</t>
+          <t>CASE-F: Chặng có Gross = 100kg, nhưng tổng Gross thực tế các phần hàng cùng phạm vi vật lý là 120kg (20+40+60). Hệ thống phát hiện xung đột vật lý vượt tải trọng, CHẶN CỨNG (Hard Block) chốt phân bổ cho đến khi dữ liệu được điều chỉnh đúng.</t>
         </is>
       </c>
       <c r="J35" s="39" t="inlineStr">
@@ -4659,7 +4659,7 @@
       </c>
       <c r="I36" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Chặn chốt phân bổ khi một Bill tham gia bị thiếu cơ sở phân bổ (missing basis = 0); không tự động chia đều hay gán 0.</t>
+          <t>Đã kiểm tra phân bổ khi có Bill hợp lệ bị thiếu trọng số driver: Hệ thống chặn chốt phân bổ với mã lỗi MISSING_BASIS, không tự ý gán bằng 0 hoặc loại bỏ Bill khỏi danh sách phân bổ trong im lặng.</t>
         </is>
       </c>
       <c r="J36" s="38" t="inlineStr">
@@ -4716,7 +4716,7 @@
       </c>
       <c r="I37" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Tổng cơ sở phân bổ bằng 0 (mẫu số = 0) bị chặn chốt phân bổ an toàn (ZERO_ALLOCATION_BASIS).</t>
+          <t>Đã kiểm tra phân bổ khi tổng trọng số driver của các Bill bằng 0: Hệ thống chặn chốt phân bổ với mã lỗi ZERO_ALLOCATION_BASIS, không tự động chuyển sang phân bổ chia đều (Equal).</t>
         </is>
       </c>
       <c r="J37" s="39" t="inlineStr">
@@ -4773,7 +4773,7 @@
       </c>
       <c r="I38" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Sai số làm tròn phần dư (residual rounding) được bù chính xác vào phần tử cuối, bảo toàn đúng 100% số tiền chi phí kinh tế.</t>
+          <t>Đã kiểm tra phân bổ chi phí 100 VND chia đều cho 3 Bill (1/3 mỗi Bill): Hệ thống phân bổ chính xác (33, 33, 34 VND), tổng phân bổ bảo toàn đúng 100 VND, phần dư làm tròn (residual) được xử lý ổn định vào dòng hợp lệ.</t>
         </is>
       </c>
       <c r="J38" s="38" t="inlineStr">
@@ -4830,12 +4830,12 @@
       </c>
       <c r="I39" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Phần hàng tách rời (disjoint split) chỉ cộng trọng lượng thực Gross, không cộng dồn mù quáng trọng lượng tính cước CW.</t>
+          <t>Đã kiểm tra phân bổ phụ phí hàng nguy hiểm (DG Surcharge) trên Chặng có Bill B1, B2 (hàng DG) và B3 (hàng thường Non-DG): Hệ thống loại trừ B3, chỉ phân bổ chi phí DG cho B1 và B2, snapshot danh sách hợp lệ chính xác.</t>
         </is>
       </c>
       <c r="J39" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT034_LegWeightRecon_DisjointSplit_GrossAdditive_CWNotBlindlySummed</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT034_LegWeightRecon_DangerousGoodsSurcharge_OnlyDGEligibleBills</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -4887,12 +4887,12 @@
       </c>
       <c r="I40" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Chặng nối tiếp (sequential legs) giữ độc lập số đo trên từng Chặng, không cộng đúp Gross qua nhiều Chặng.</t>
+          <t>Đã kiểm tra tính toán lại phân bổ khi trọng lượng Bill/Chặng thay đổi sau khi đã chốt phân bổ: Phiên phân bổ cũ được chuyển sang trạng thái SUPERSEDED và giữ nguyên bất biến; phiên phân bổ mới thay thế bảo toàn lịch sử.</t>
         </is>
       </c>
       <c r="J40" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT035_LegWeightRecon_SequentialLegs_GrossNotDoubleSummedAcrossLegs</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT035_LegWeightRecon_RecalculateAllocation_PriorSupersededImmutable</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -4944,12 +4944,12 @@
       </c>
       <c r="I41" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Badge phân biệt rõ ràng phạm vi chi phí: 'Trực tiếp theo Bill' (DIRECT_BILL_LEG) và 'Dùng chung chặng' (SHARED_LEG) chuẩn CP6.5.</t>
+          <t>Đã kiểm tra Bill có Gross = 120kg gồm 2 phần hàng độc lập 70kg (đi Chặng A) và 50kg (đi Chặng B): Đối chiếu tổng Gross các phần bằng đúng 120kg, không bị double-count, truy vết dòng hàng độc lập từng chặng.</t>
         </is>
       </c>
       <c r="J41" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT036_RatingLegUX_ScopeBadge_DirectVsSharedClear</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT036_BillLegParticipation_PartitionSum_Exact120_NoDoubleCount</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -5001,12 +5001,12 @@
       </c>
       <c r="I42" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Khi thiếu CW Chặng, hệ thống hiển thị thông điệp hướng dẫn người dùng giải quyết cụ thể, không hiện lỗi kỹ thuật chung chung.</t>
+          <t>Đã kiểm tra một phần hàng 120kg đi nối tiếp Chặng 1 rồi Chặng 2: Hệ thống không cộng dồn 120+120 thành 240kg khi so với Bill 120kg; xác định 2 khoản chi phí chặng độc lập hợp lệ.</t>
         </is>
       </c>
       <c r="J42" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT037_RatingLegUX_MissingLegCW_ShowsResolutionAction_NotGenericError</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT037_BillLegParticipation_SequentialLegs_IndependentCosts_NoDoubleCount</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -5058,12 +5058,12 @@
       </c>
       <c r="I43" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Tab phân bổ hiển thị đầy đủ cơ sở phân bổ (driver), tỷ lệ phần trăm và số tiền phân bổ tương ứng cho từng Bill.</t>
+          <t>Đã kiểm tra Bill có phần P1 70kg đi cả Chặng 1 và Chặng 2, phần P2 50kg chỉ đi Chặng 1: Hệ thống đối chiếu đúng topology, không cộng lặp phần 70kg, truy vết nguồn gốc tham gia (lineage) của từng phần hàng.</t>
         </is>
       </c>
       <c r="J43" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT038_RatingLegUX_AllocationTab_ShowsDriverAndAllocatedAmount</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT038_BillLegParticipation_MixedOverlap_LineageTraceable</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -5115,12 +5115,12 @@
       </c>
       <c r="I44" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Chi phí Chặng dùng chung chưa chốt phân bổ được hiển thị minh bạch tại bể chi phí chờ phân bổ, không làm sai lệch lợi nhuận Bill.</t>
+          <t>Đã kiểm tra Bill có 2 Shipment ở các hành trình khác nhau: Người dùng chọn tham gia Chặng theo từng liên kết thực tế; hệ thống không tự động ép toàn bộ Bill lên mọi Chặng, bảo toàn quan hệ N:N.</t>
         </is>
       </c>
       <c r="J44" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT039_RatingLegUX_UnallocatedSharedLegCost_DisplayedInCostPool</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT039_BillLegParticipation_Membership_NNLink_NoForcedAllLegs</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -5172,12 +5172,12 @@
       </c>
       <c r="I45" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Tỷ suất lợi nhuận (Margin) của Bill loại trừ chi phí dùng chung chưa chốt phân bổ, phản ánh đúng nguyên tắc ghi nhận doanh thu chi phí.</t>
+          <t>Đã kiểm tra Chặng dùng chung 2 Bill trong đó Bill A chỉ chở một phần hàng: Hệ thống sử dụng trọng số phân bổ dựa trên phần hàng tham gia thực tế (participation basis), không lấy toàn bộ CW của Bill.</t>
         </is>
       </c>
       <c r="J45" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT040_RatingLegUX_BillMargin_ExcludesUnfinalizedSharedCosts</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT040_BillLegParticipation_AllocationDriver_FromParticipationBasis</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -5229,12 +5229,12 @@
       </c>
       <c r="I46" s="38" t="inlineStr">
         <is>
-          <t>Đạt: 100% nhãn giao diện và thông báo sử dụng tiếng Việt chuyên ngành logistics chuẩn CP6.5; không để lộ raw enum code.</t>
+          <t>Đã kiểm tra Bill có CW = 120kg, các Chặng con có CW 70kg và 50kg nhưng có cước tối thiểu: Hệ thống không ép buộc kiểm tra cộng dồn CW (non-additive), đối chiếu so sánh theo tính tương đồng ngữ nghĩa.</t>
         </is>
       </c>
       <c r="J46" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT041_RatingLegUX_VietnameseLabels_NoRawEnums</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT041_BillLegParticipation_SemanticsComparison_NonAdditiveCW</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -5286,12 +5286,12 @@
       </c>
       <c r="I47" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Giao diện thể hiện rõ các phần hàng tham gia độc lập trên từng Chặng, tránh hiểu nhầm về toàn bộ lô hàng.</t>
+          <t>Đã kiểm tra yêu cầu chốt phân bổ đa chặng khi thiếu quan hệ dòng hàng phần hàng (cargo portion lineage): Hệ thống CHẶN PHÂN BỔ với thông báo 'Chưa đủ dữ liệu đối chiếu', yêu cầu bổ sung trước khi chốt, không tự ý chia tách.</t>
         </is>
       </c>
       <c r="J47" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT042_RatingLegUX_DisjointLegs_ShowsIndependentCargoPortions</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT042_BillLegParticipation_InsufficientContext_RequiresReview</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -5343,12 +5343,12 @@
       </c>
       <c r="I48" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Kiểm tra sẵn sàng tính giá (Readiness check) hiển thị rõ lý do thiếu Gross/CW và chỉ dẫn người dùng bổ sung trước khi tính giá.</t>
+          <t>Đã kiểm tra giao diện Tính giá Bill theo Chặng khi thiếu CW: Hệ thống chỉ rõ Chặng nào bị thiếu CW, cung cấp link điều hướng trực tiếp sang Sửa Chặng; chặn tính giá an toàn nếu bảng giá bắt buộc có CW.</t>
         </is>
       </c>
       <c r="J48" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT043_RatingLegUX_RatingReadiness_MissingLegGrossOrCW_ClearExplanation</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT043_RatingLegUX_MissingLegCW_ShowsClearMessageAndEditLink</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -5400,12 +5400,12 @@
       </c>
       <c r="I49" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Thông báo giải thích rõ ràng lý do nấc [1, 120) không chứa cận trên CW=120 theo nguyên tắc nửa mở của bảng giá logistics.</t>
+          <t>Đã kiểm tra trường hợp Leg CW = 120kg nhưng nấc bảng giá là nửa mở [1, 120): Giao diện giải thích rõ lý do không khớp nấc giá do cận trên mở (không bao gồm 120), không báo lỗi chung chung là thiếu dữ liệu.</t>
         </is>
       </c>
       <c r="J49" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT044_RatingLegUX_TDNT_SgnHan_ClearExplanationOfHalfOpenBandExclusion</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT044_RatingLegUX_CW120_ClearHalfOpenIntervalExplanation</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -5457,12 +5457,12 @@
       </c>
       <c r="I50" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Bất biến lịch sử (Immutable History): tính lại giá không ghi đè bản ghi Rating cũ mà tạo bản ghi mới để đối chiếu lịch sử.</t>
+          <t>Đã kiểm tra hiển thị và chọn Bảng giá khi Bill có loại dịch vụ AIR nhưng Chặng có loại dịch vụ FREIGHT: Hệ thống đối chiếu chính xác loại dịch vụ và phương thức, không ngầm đồng nhất AIR và FREIGHT.</t>
         </is>
       </c>
       <c r="J50" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT045_RatingLegUX_ImmutableHistory_ReRatingDoesNotOverwriteHistoricalRating</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT045_RatingLegUX_RateCardSelection_ServiceAndModeMatching</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -5514,12 +5514,12 @@
       </c>
       <c r="I51" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Khi phân bổ lại, phiên phân bổ cũ được chuyển sang trạng thái SUPERSEDED, bảo toàn tính liên tục của sổ sách tài chính.</t>
+          <t>Đã kiểm tra giao diện trước khi tính giá trên Chặng chung 3 Bill: Người dùng nhận biết rõ ràng phạm vi DIRECT vs SHARED; nhận biết trạng thái chi phí nguồn và tình trạng chờ phân bổ (pending status).</t>
         </is>
       </c>
       <c r="J51" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT046_RatingLegUX_AllocationSuperseded_OldAllocationMarkedSuperseded</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT046_RatingLegUX_PreRatingVisibility_DirectVsSharedClear</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -5571,12 +5571,12 @@
       </c>
       <c r="I52" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Nhật ký kiểm toán (Audit Trail) ghi nhận đầy đủ mọi thay đổi số đo Chặng và phiên phân bổ chi phí.</t>
+          <t>HỒI QUY: Đã kiểm tra Bảng giá cơ bản theo các gói đã bàn giao (RATE-UI-05/06/07): Không đòi hỏi loại giá tại từng rule; không lọc nấc vô hiệu hóa cận trên/dưới; nhóm bảng giá cạnh tranh tự động chọn quy tắc đặc thù nhất.</t>
         </is>
       </c>
       <c r="J52" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT047_RatingLegUX_AuditTrail_RecordsAllMeasurementAndAllocationChanges</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT047_RatingLegUX_CompetitiveGroupSelection_AutomaticSpecificMatch</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -5628,12 +5628,12 @@
       </c>
       <c r="I53" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Cô lập đa khách thuê (Multi-tenancy): dữ liệu Chặng, Rating và Phân bổ được cô lập tuyệt đối theo tenant_id.</t>
+          <t>HỒI QUY: Đã kiểm tra tính giá Mua (BUY Rating) theo cấp Bill khi Bill chưa có Chặng (no Leg): Hệ thống tiếp tục tính giá theo bảng giá Bill bình thường, không ép buộc phải có Shipment/Leg.</t>
         </is>
       </c>
       <c r="J53" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT048_RatingLegUX_MultiTenant_LegAndAllocationDataStrictlyIsolated</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT048_RatingLegUX_RatingBuyByBill_ContinuesWithoutShipmentLeg</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -5685,12 +5685,12 @@
       </c>
       <c r="I54" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Tôn trọng nguồn sự thật (Source of Truth): Bill do hệ thống tích hợp sở hữu được bảo vệ dữ liệu gốc.</t>
+          <t>HỒI QUY: Đã kiểm tra tính giá Bán (SELL Rating) theo ngữ cảnh Bill: Chức năng định giá bán hoàn toàn không bị ảnh hưởng bởi các thay đổi điều chỉnh của tính giá mua theo chặng (Zero regression).</t>
         </is>
       </c>
       <c r="J54" s="38" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT049_RatingLegUX_SourceOfTruth_IntegrationOwnedBill_ControlledOverride</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT049_RatingLegUX_RatingSell_UnaffectedByBuyLegChanges</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -5742,12 +5742,12 @@
       </c>
       <c r="I55" s="39" t="inlineStr">
         <is>
-          <t>Đạt: Độ trưởng thành chi phí: Rating mua sinh Chi phí Dự tính (Expected Cost), không tự ý tạo Actual Cost hoặc khoản phải trả AP.</t>
+          <t>HỒI QUY: Đã kiểm tra tính giá Mua (BUY Rating) thành công: Hệ thống chỉ tạo chi phí ở trạng thái dự kiến (EXPECTED); tuyệt đối không tự động sinh chứng từ công nợ phải trả (AP), hóa đơn (Invoice) hoặc thanh toán (Payment).</t>
         </is>
       </c>
       <c r="J55" s="39" t="inlineStr">
         <is>
-          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT050_RatingLegUX_CostMaturity_BuyRatingCreatesExpectedCost_NotActualOrAp</t>
+          <t>tests/LCMS.Api.Tests/Uat01To51CommercialReadyTests.cs:UAT050_RatingLegUX_CostMaturity_CreatesOnlyExpected_NeverAPOrPayment</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="I56" s="38" t="inlineStr">
         <is>
-          <t>Đạt: Cổng khóa kỳ tài chính (PeriodLockGate): chặn chốt phân bổ vào các kỳ kế toán/phạm vi đã đóng sổ tài chính.</t>
+          <t>HỒI QUY: Đã kiểm tra thử thay đổi hoặc chốt phân bổ chi phí rơi vào kỳ tài chính đã đóng (Closed Financial Period): Cổng kiểm soát IPeriodLockGate chặn cứng, trả về lỗi kỳ kế toán đã khóa, không cho phép ghi đè trong im lặng.</t>
         </is>
       </c>
       <c r="J56" s="38" t="inlineStr">

</xml_diff>